<commit_message>
Fix positive test data: add DTHDTC for CDISC005 in dm.xpt
</commit_message>
<xml_diff>
--- a/rules/CORE-000841/positive/01/data/unit-test-coreid-FB0612-positive.xlsx
+++ b/rules/CORE-000841/positive/01/data/unit-test-coreid-FB0612-positive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulieChason\GitHub\core-contributor\rules\CORE-000841\positive\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F504C17-4A7F-4AD5-9194-C1B73E9E778B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{339E4741-736C-4182-924C-8A285F5C6338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="9772" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="124">
   <si>
     <t>Product</t>
   </si>
@@ -487,7 +487,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -522,16 +522,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1698,79 +1691,79 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:26" s="17" customFormat="1" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:26" ht="58.3" x14ac:dyDescent="0.4">
+      <c r="A6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="11">
         <v>1211</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="J6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="K6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="14" t="s">
+      <c r="L6" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="M6" s="15">
+      <c r="M6" s="11">
         <v>701</v>
       </c>
-      <c r="N6" s="15">
+      <c r="N6" s="11">
         <v>1955</v>
       </c>
-      <c r="O6" s="14" t="s">
+      <c r="O6" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="P6" s="14" t="s">
+      <c r="P6" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="Q6" s="14" t="s">
+      <c r="Q6" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="R6" s="14" t="s">
+      <c r="R6" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="S6" s="14" t="s">
+      <c r="S6" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="T6" s="14" t="s">
+      <c r="T6" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="U6" s="14" t="s">
+      <c r="U6" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="V6" s="14" t="s">
+      <c r="V6" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="W6" s="14" t="s">
+      <c r="W6" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="X6" s="14"/>
-      <c r="Y6" s="14"/>
-      <c r="Z6" s="14" t="s">
+      <c r="X6" s="9"/>
+      <c r="Y6" s="9"/>
+      <c r="Z6" s="9" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1943,7 +1936,7 @@
       <c r="F9" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="16" t="s">
         <v>121</v>
       </c>
       <c r="H9" s="10" t="s">
@@ -1955,7 +1948,9 @@
       <c r="J9" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="K9" s="10"/>
+      <c r="K9" s="10" t="s">
+        <v>120</v>
+      </c>
       <c r="L9" s="9"/>
       <c r="M9" s="11">
         <v>701</v>
@@ -1997,157 +1992,157 @@
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
     </row>
     <row r="17" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
     </row>
     <row r="18" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
     </row>
     <row r="19" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
     </row>
     <row r="20" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
     </row>
     <row r="21" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
     </row>
     <row r="22" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
     </row>
     <row r="23" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
     </row>
     <row r="24" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
     </row>
     <row r="25" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
     </row>
     <row r="26" spans="5:11" x14ac:dyDescent="0.4">
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="18"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>